<commit_message>
Add classification model, access workflow, minimum necessary policy, and access workbooks
</commit_message>
<xml_diff>
--- a/05_access_and_privacy/access-control-matrix.xlsx
+++ b/05_access_and_privacy/access-control-matrix.xlsx
@@ -8,15 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Documents\GitHub\enterprise-data-governance-operating-system\05_access_and_privacy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EE954D95-484F-4522-9462-D4DC444F97AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AAD2E02-562A-418D-A42C-9C89E34C71ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="22695" windowHeight="14476" xr2:uid="{17F23537-A27D-40DF-B066-E18384E7CF1B}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="22695" windowHeight="14476" activeTab="1" xr2:uid="{17F23537-A27D-40DF-B066-E18384E7CF1B}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="3" r:id="rId1"/>
     <sheet name="Access Matrix" sheetId="2" r:id="rId2"/>
     <sheet name="Roles" sheetId="1" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Access Matrix'!$A$1:$L$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Roles!$A$1:$D$7</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -38,11 +42,278 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="82">
+  <si>
+    <t>Access Control Matrix Workbook</t>
+  </si>
+  <si>
+    <t>Purpose</t>
+  </si>
+  <si>
+    <t>Maps typical access rights by role, asset class, and action type to support minimum-necessary access design.</t>
+  </si>
+  <si>
+    <t>How to use</t>
+  </si>
+  <si>
+    <t>Use one row per role-to-asset pattern. Confirm default access, approval path, and conditions before implementation.</t>
+  </si>
+  <si>
+    <t>Governance rule</t>
+  </si>
+  <si>
+    <t>Broad access, sensitive assets, and export rights should require stronger review and clear rationale.</t>
+  </si>
+  <si>
+    <t>Role</t>
+  </si>
+  <si>
+    <t>Typical Need</t>
+  </si>
+  <si>
+    <t>Default Access Posture</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Executive Viewer</t>
+  </si>
+  <si>
+    <t>High-level certified reporting</t>
+  </si>
+  <si>
+    <t>Read-only, aggregated</t>
+  </si>
+  <si>
+    <t>Usually no source-level access</t>
+  </si>
+  <si>
+    <t>Manager</t>
+  </si>
+  <si>
+    <t>Operational and management reporting</t>
+  </si>
+  <si>
+    <t>Read-only plus limited drill-down</t>
+  </si>
+  <si>
+    <t>Scope should match business unit</t>
+  </si>
+  <si>
+    <t>Analyst</t>
+  </si>
+  <si>
+    <t>Detailed analysis and recurring reporting</t>
+  </si>
+  <si>
+    <t>Read-only to approved layers, limited source access where justified</t>
+  </si>
+  <si>
+    <t>Avoid default full-system rights</t>
+  </si>
+  <si>
+    <t>Data Steward</t>
+  </si>
+  <si>
+    <t>Metadata, issue, and access coordination</t>
+  </si>
+  <si>
+    <t>Read-only plus workflow support access</t>
+  </si>
+  <si>
+    <t>Not automatically the business approver</t>
+  </si>
+  <si>
+    <t>System Administrator</t>
+  </si>
+  <si>
+    <t>Technical administration</t>
+  </si>
+  <si>
+    <t>Elevated technical access</t>
+  </si>
+  <si>
+    <t>Should not replace business approval</t>
+  </si>
+  <si>
+    <t>External Partner</t>
+  </si>
+  <si>
+    <t>Approved narrow-purpose exchange</t>
+  </si>
+  <si>
+    <t>Exception-based, time-bound</t>
+  </si>
+  <si>
+    <t>Usually highly restricted</t>
+  </si>
+  <si>
+    <t>Asset / System</t>
+  </si>
+  <si>
+    <t>Asset Classification</t>
+  </si>
+  <si>
+    <t>Access Scope</t>
+  </si>
+  <si>
+    <t>Read</t>
+  </si>
+  <si>
+    <t>Edit</t>
+  </si>
+  <si>
+    <t>Export</t>
+  </si>
+  <si>
+    <t>Share</t>
+  </si>
+  <si>
+    <t>Approval Required</t>
+  </si>
+  <si>
+    <t>Decision Owner</t>
+  </si>
+  <si>
+    <t>Review Frequency</t>
+  </si>
+  <si>
+    <t>Conditions / Notes</t>
+  </si>
+  <si>
+    <t>Certified KPI Dashboard</t>
+  </si>
+  <si>
+    <t>Internal</t>
+  </si>
+  <si>
+    <t>Aggregated certified view</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Limited</t>
+  </si>
+  <si>
+    <t>Standard</t>
+  </si>
+  <si>
+    <t>Reporting Director</t>
+  </si>
+  <si>
+    <t>Quarterly</t>
+  </si>
+  <si>
+    <t>No direct source access</t>
+  </si>
+  <si>
+    <t>Operational Performance Report</t>
+  </si>
+  <si>
+    <t>Business-unit scoped</t>
+  </si>
+  <si>
+    <t>Business Owner</t>
+  </si>
+  <si>
+    <t>Scope aligned to operating unit</t>
+  </si>
+  <si>
+    <t>Reporting Mart</t>
+  </si>
+  <si>
+    <t>Confidential</t>
+  </si>
+  <si>
+    <t>Detailed approved layer</t>
+  </si>
+  <si>
+    <t>Controlled</t>
+  </si>
+  <si>
+    <t>Owner approval</t>
+  </si>
+  <si>
+    <t>Data Owner</t>
+  </si>
+  <si>
+    <t>Export subject to business purpose</t>
+  </si>
+  <si>
+    <t>Glossary and Issue Logs</t>
+  </si>
+  <si>
+    <t>Governance artifacts</t>
+  </si>
+  <si>
+    <t>Governance Lead</t>
+  </si>
+  <si>
+    <t>Workflow support only</t>
+  </si>
+  <si>
+    <t>Access Provisioning Console</t>
+  </si>
+  <si>
+    <t>Restricted</t>
+  </si>
+  <si>
+    <t>Technical admin scope</t>
+  </si>
+  <si>
+    <t>Manager plus control</t>
+  </si>
+  <si>
+    <t>System Owner</t>
+  </si>
+  <si>
+    <t>Technical administration only</t>
+  </si>
+  <si>
+    <t>Approved Extract</t>
+  </si>
+  <si>
+    <t>Narrow approved subset</t>
+  </si>
+  <si>
+    <t>Exception approval</t>
+  </si>
+  <si>
+    <t>Per request</t>
+  </si>
+  <si>
+    <t>Time-bound and purpose-bound</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -69,8 +340,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -385,27 +658,450 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AFAF8F4-2DBA-4639-8B43-B0813B214AD1}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="34.9296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="93.86328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="135" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8927AA91-7050-4CEB-A6CF-9C7F7F6C0BBD}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="17.86328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.46484375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.59765625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.9296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.53125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.265625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.86328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.86328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="28.19921875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G2" t="s">
+        <v>51</v>
+      </c>
+      <c r="H2" t="s">
+        <v>50</v>
+      </c>
+      <c r="I2" t="s">
+        <v>52</v>
+      </c>
+      <c r="J2" t="s">
+        <v>53</v>
+      </c>
+      <c r="K2" t="s">
+        <v>54</v>
+      </c>
+      <c r="L2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E3" t="s">
+        <v>49</v>
+      </c>
+      <c r="F3" t="s">
+        <v>50</v>
+      </c>
+      <c r="G3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H3" t="s">
+        <v>50</v>
+      </c>
+      <c r="I3" t="s">
+        <v>52</v>
+      </c>
+      <c r="J3" t="s">
+        <v>58</v>
+      </c>
+      <c r="K3" t="s">
+        <v>54</v>
+      </c>
+      <c r="L3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E4" t="s">
+        <v>49</v>
+      </c>
+      <c r="F4" t="s">
+        <v>50</v>
+      </c>
+      <c r="G4" t="s">
+        <v>63</v>
+      </c>
+      <c r="H4" t="s">
+        <v>50</v>
+      </c>
+      <c r="I4" t="s">
+        <v>64</v>
+      </c>
+      <c r="J4" t="s">
+        <v>65</v>
+      </c>
+      <c r="K4" t="s">
+        <v>54</v>
+      </c>
+      <c r="L4" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D5" t="s">
+        <v>68</v>
+      </c>
+      <c r="E5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G5" t="s">
+        <v>51</v>
+      </c>
+      <c r="H5" t="s">
+        <v>50</v>
+      </c>
+      <c r="I5" t="s">
+        <v>52</v>
+      </c>
+      <c r="J5" t="s">
+        <v>69</v>
+      </c>
+      <c r="K5" t="s">
+        <v>54</v>
+      </c>
+      <c r="L5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" t="s">
+        <v>71</v>
+      </c>
+      <c r="C6" t="s">
+        <v>72</v>
+      </c>
+      <c r="D6" t="s">
+        <v>73</v>
+      </c>
+      <c r="E6" t="s">
+        <v>49</v>
+      </c>
+      <c r="F6" t="s">
+        <v>49</v>
+      </c>
+      <c r="G6" t="s">
+        <v>50</v>
+      </c>
+      <c r="H6" t="s">
+        <v>50</v>
+      </c>
+      <c r="I6" t="s">
+        <v>74</v>
+      </c>
+      <c r="J6" t="s">
+        <v>75</v>
+      </c>
+      <c r="K6" t="s">
+        <v>54</v>
+      </c>
+      <c r="L6" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" t="s">
+        <v>77</v>
+      </c>
+      <c r="C7" t="s">
+        <v>72</v>
+      </c>
+      <c r="D7" t="s">
+        <v>78</v>
+      </c>
+      <c r="E7" t="s">
+        <v>49</v>
+      </c>
+      <c r="F7" t="s">
+        <v>50</v>
+      </c>
+      <c r="G7" t="s">
+        <v>63</v>
+      </c>
+      <c r="H7" t="s">
+        <v>50</v>
+      </c>
+      <c r="I7" t="s">
+        <v>79</v>
+      </c>
+      <c r="J7" t="s">
+        <v>65</v>
+      </c>
+      <c r="K7" t="s">
+        <v>80</v>
+      </c>
+      <c r="L7" t="s">
+        <v>81</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:L7" xr:uid="{8927AA91-7050-4CEB-A6CF-9C7F7F6C0BBD}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CAC564B-CE59-4AC6-A711-F1EFBFDCADAB}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="17.86328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="33.3984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="54.06640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="32.86328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D7" xr:uid="{0CAC564B-CE59-4AC6-A711-F1EFBFDCADAB}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>